<commit_message>
deploy: main → 7497e47552ea2cee611c58d0b7b6fa7120287707
</commit_message>
<xml_diff>
--- a/StructureDefinition-IneraPatient.xlsx
+++ b/StructureDefinition-IneraPatient.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.1</t>
+    <t>1.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-24T17:45:04+00:00</t>
+    <t>2026-06-25T07:04:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → 9a87c56f6f5a4637b3a120f6e3e6038fff29dff2
</commit_message>
<xml_diff>
--- a/StructureDefinition-IneraPatient.xlsx
+++ b/StructureDefinition-IneraPatient.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-25T07:50:33+00:00</t>
+    <t>2026-06-25T07:55:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
deploy: main → 4f5b70ce186e216fb00d9e54ef16cadd30f40d47
</commit_message>
<xml_diff>
--- a/StructureDefinition-IneraPatient.xlsx
+++ b/StructureDefinition-IneraPatient.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0</t>
+    <t>2.1.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-14T09:00:12+00:00</t>
+    <t>2026-07-14T13:33:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>